<commit_message>
Update sample Excel with user phone numbers 9584510000, 8889888034, 8839250427
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>Rahul Sharma</v>
       </c>
       <c r="B2" t="str">
-        <v>918839250427</v>
+        <v>919584510000</v>
       </c>
       <c r="C2" t="str">
         <v>CA Inter IDT Full Book Set 8.0</v>
@@ -452,7 +452,7 @@
         <v>Priya Patel</v>
       </c>
       <c r="B3" t="str">
-        <v>917746875564</v>
+        <v>918889888034</v>
       </c>
       <c r="C3" t="str">
         <v>CA Final Tax Fast Track Book</v>
@@ -465,11 +465,31 @@
       </c>
       <c r="F3" t="str">
         <v>DTDC Courier</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Garv Joshi</v>
+      </c>
+      <c r="B4" t="str">
+        <v>918839250427</v>
+      </c>
+      <c r="C4" t="str">
+        <v>CA Foundation Accounting Module</v>
+      </c>
+      <c r="D4" t="str">
+        <v>BLR123456789</v>
+      </c>
+      <c r="E4" t="str">
+        <v>03-10-2026</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Blue Dart</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Excel template with all 6 user phone numbers
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F7"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -432,7 +432,7 @@
         <v>Rahul Sharma</v>
       </c>
       <c r="B2" t="str">
-        <v>919584510000</v>
+        <v>919669011750</v>
       </c>
       <c r="C2" t="str">
         <v>CA Inter IDT Full Book Set 8.0</v>
@@ -452,7 +452,7 @@
         <v>Priya Patel</v>
       </c>
       <c r="B3" t="str">
-        <v>918889888034</v>
+        <v>918103554325</v>
       </c>
       <c r="C3" t="str">
         <v>CA Final Tax Fast Track Book</v>
@@ -487,9 +487,69 @@
         <v>Blue Dart</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Ankit Verma</v>
+      </c>
+      <c r="B5" t="str">
+        <v>917746875564</v>
+      </c>
+      <c r="C5" t="str">
+        <v>CA Inter Law Study Material</v>
+      </c>
+      <c r="D5" t="str">
+        <v>C1144019999IN</v>
+      </c>
+      <c r="E5" t="str">
+        <v>03-10-2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>India Post</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Neha Singh</v>
+      </c>
+      <c r="B6" t="str">
+        <v>919584510000</v>
+      </c>
+      <c r="C6" t="str">
+        <v>CA Final Audit Crush Book</v>
+      </c>
+      <c r="D6" t="str">
+        <v>DT88887777IN</v>
+      </c>
+      <c r="E6" t="str">
+        <v>03-10-2026</v>
+      </c>
+      <c r="F6" t="str">
+        <v>DTDC Courier</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Amit Kumar</v>
+      </c>
+      <c r="B7" t="str">
+        <v>918889888034</v>
+      </c>
+      <c r="C7" t="str">
+        <v>CA Inter Costing Fast Track</v>
+      </c>
+      <c r="D7" t="str">
+        <v>BLR99998888</v>
+      </c>
+      <c r="E7" t="str">
+        <v>03-10-2026</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Blue Dart</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>